<commit_message>
content: HFA default indicators: code columns drop R's name
The platform's workbook import now reads code__<time point>,
filter_code__<time point> and variant_code__<item id>__<time point>, and
refuses the old r_code__ headers. Only the five header cells of the
Indicators sheet changed; every other cell and every other part of the file
is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hfa_default_indicators.xlsx
+++ b/hfa_default_indicators.xlsx
@@ -781,19 +781,19 @@
         <v>variantGroupId</v>
       </c>
       <c r="M1" t="str">
-        <v>r_code__Round 1</v>
+        <v>code__Round 1</v>
       </c>
       <c r="N1" t="str">
-        <v>r_filter_code__Round 1</v>
+        <v>filter_code__Round 1</v>
       </c>
       <c r="O1" t="str">
-        <v>r_variant_code__mobile_strategy__Round 1</v>
+        <v>variant_code__mobile_strategy__Round 1</v>
       </c>
       <c r="P1" t="str">
-        <v>r_variant_code__fixed_strategy__Round 1</v>
+        <v>variant_code__fixed_strategy__Round 1</v>
       </c>
       <c r="Q1" t="str">
-        <v>r_variant_code__mobile_and_fixed_strategy__Round 1</v>
+        <v>variant_code__mobile_and_fixed_strategy__Round 1</v>
       </c>
     </row>
     <row r="2">

</xml_diff>